<commit_message>
sys id test results
</commit_message>
<xml_diff>
--- a/HIVE/relay/info/xbee_info.xlsx
+++ b/HIVE/relay/info/xbee_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\all my files\documents\uvm\5_masters\hive\github_directory\HIVE\relay\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074ADC7D-C10A-4C0C-A318-1E08726A5843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6625E646-4E3E-4EDE-AA0C-60C2EB82F14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4590" yWindow="16080" windowWidth="29040" windowHeight="15840" xr2:uid="{811B69A6-7BAA-47F7-8449-D6A98DB96D93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{811B69A6-7BAA-47F7-8449-D6A98DB96D93}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,6 +39,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={9CEBB753-356C-4B05-92F4-85D18BBE23D9}</author>
+    <author>tc={EC338FC7-A91D-4B88-8C83-FB76E889FF08}</author>
   </authors>
   <commentList>
     <comment ref="A3" authorId="0" shapeId="0" xr:uid="{9CEBB753-356C-4B05-92F4-85D18BBE23D9}">
@@ -46,10 +47,15 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Setup as:
-coord: 1
-end:     3
-rout:    2,4</t>
+    Setup as fixed chain 1-&gt;2-&gt;4-&gt;5</t>
+      </text>
+    </comment>
+    <comment ref="A5" authorId="1" shapeId="0" xr:uid="{EC338FC7-A91D-4B88-8C83-FB76E889FF08}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not behaving</t>
       </text>
     </comment>
   </commentList>
@@ -57,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -216,13 +222,19 @@
   </si>
   <si>
     <t>99_router</t>
+  </si>
+  <si>
+    <t>40D5B2B4</t>
+  </si>
+  <si>
+    <t>xbee_5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -230,16 +242,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -247,18 +277,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="23">
@@ -357,10 +410,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8266905B-4801-4118-B402-E0A40CDD2BC9}" name="Table1" displayName="Table1" ref="A2:U15" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A2:U15" xr:uid="{8266905B-4801-4118-B402-E0A40CDD2BC9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:U11">
-    <sortCondition ref="A2:A15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8266905B-4801-4118-B402-E0A40CDD2BC9}" name="Table1" displayName="Table1" ref="A2:U17" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A2:U17" xr:uid="{8266905B-4801-4118-B402-E0A40CDD2BC9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:U17">
+    <sortCondition ref="A2:A17"/>
   </sortState>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{C23D5EF9-DF7F-4225-85F1-8152BF153E54}" name="ID" dataDxfId="20"/>
@@ -707,17 +760,17 @@
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="A3" dT="2024-12-04T18:28:49.34" personId="{63701861-AAD2-4F9A-AA46-A629DA70D705}" id="{9CEBB753-356C-4B05-92F4-85D18BBE23D9}">
-    <text>Setup as:
-coord: 1
-end:     3
-rout:    2,4</text>
+    <text>Setup as fixed chain 1-&gt;2-&gt;4-&gt;5</text>
+  </threadedComment>
+  <threadedComment ref="A5" dT="2024-12-23T17:13:05.39" personId="{63701861-AAD2-4F9A-AA46-A629DA70D705}" id="{EC338FC7-A91D-4B88-8C83-FB76E889FF08}">
+    <text>Not behaving</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C958D8FD-ED38-4072-847E-9B96E34E794A}">
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -725,7 +778,7 @@
     <col min="3" max="5" width="9.140625" style="1"/>
     <col min="6" max="6" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="9.140625" style="1"/>
-    <col min="9" max="9" width="19.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.7109375" style="1" customWidth="1"/>
     <col min="11" max="12" width="9.140625" style="1"/>
     <col min="13" max="14" width="9.140625" style="1" customWidth="1"/>
@@ -735,28 +788,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2" t="s">
+      <c r="F1" s="4"/>
+      <c r="G1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="2"/>
-      <c r="M1" s="2" t="s">
+      <c r="H1" s="4"/>
+      <c r="M1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2" t="s">
+      <c r="N1" s="4"/>
+      <c r="O1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2" t="s">
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -842,11 +895,11 @@
       <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="1">
-        <v>0</v>
-      </c>
-      <c r="H3" s="1">
-        <v>0</v>
+      <c r="G3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>15</v>
@@ -904,11 +957,11 @@
       <c r="F4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="1">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0</v>
+      <c r="G4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>15</v>
@@ -947,32 +1000,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>3332</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="J5" s="1">
@@ -1028,6 +1081,12 @@
       <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="G6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>53</v>
+      </c>
       <c r="I6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1067,46 +1126,40 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="1">
-        <v>14</v>
+        <v>44</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="D7" s="1">
-        <v>2015</v>
+        <v>3332</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
       </c>
-      <c r="K7" s="1">
-        <v>1</v>
-      </c>
       <c r="L7" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="M7" s="1">
         <v>4</v>
       </c>
+      <c r="N7" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="O7" s="1">
         <v>0</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>36</v>
+      <c r="P7" s="1">
+        <v>0</v>
       </c>
       <c r="Q7" s="1">
         <v>38400</v>
@@ -1126,7 +1179,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>43</v>
@@ -1141,7 +1194,7 @@
         <v>8</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G8" s="1">
         <v>0</v>
@@ -1156,7 +1209,7 @@
         <v>1</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M8" s="1">
         <v>4</v>
@@ -1185,74 +1238,74 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="C9" s="1">
+        <v>14</v>
+      </c>
+      <c r="D9" s="1">
+        <v>2015</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1">
+        <v>1</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="M9" s="1">
+        <v>4</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>38400</v>
+      </c>
+      <c r="R9" s="1">
+        <v>0</v>
+      </c>
+      <c r="S9" s="1">
+        <v>3</v>
+      </c>
+      <c r="T9" s="1">
+        <v>0</v>
+      </c>
+      <c r="U9" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="C10" s="1">
-        <v>14</v>
-      </c>
-      <c r="D10" s="1">
-        <v>2015</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="J10" s="1">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1">
-        <v>0</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="M10" s="1">
-        <v>4</v>
-      </c>
-      <c r="O10" s="1">
-        <v>0</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>38400</v>
-      </c>
-      <c r="R10" s="1">
-        <v>0</v>
-      </c>
-      <c r="S10" s="1">
-        <v>3</v>
-      </c>
-      <c r="T10" s="1">
-        <v>0</v>
-      </c>
-      <c r="U10" s="1">
-        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>42</v>
@@ -1267,7 +1320,7 @@
         <v>8</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G11" s="1">
         <v>0</v>
@@ -1276,19 +1329,19 @@
         <v>0</v>
       </c>
       <c r="J11" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M11" s="1">
         <v>4</v>
       </c>
       <c r="O11" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>36</v>
@@ -1306,12 +1359,12 @@
         <v>0</v>
       </c>
       <c r="U11" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>42</v>
@@ -1325,6 +1378,9 @@
       <c r="E12" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="F12" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="G12" s="1">
         <v>0</v>
       </c>
@@ -1338,13 +1394,13 @@
         <v>1</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="M12" s="1">
         <v>4</v>
       </c>
       <c r="O12" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P12" s="1" t="s">
         <v>36</v>
@@ -1362,12 +1418,12 @@
         <v>0</v>
       </c>
       <c r="U12" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>42</v>
@@ -1394,7 +1450,7 @@
         <v>1</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="M13" s="1">
         <v>4</v>
@@ -1423,67 +1479,126 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>42</v>
+      </c>
+      <c r="C14" s="1">
+        <v>14</v>
+      </c>
+      <c r="D14" s="1">
+        <v>2015</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M14" s="1">
+        <v>4</v>
+      </c>
+      <c r="O14" s="1">
+        <v>0</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>38400</v>
+      </c>
+      <c r="R14" s="1">
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
+        <v>3</v>
+      </c>
+      <c r="T14" s="1">
+        <v>0</v>
+      </c>
+      <c r="U14" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1">
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>99</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="1">
         <v>14</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D16" s="1">
         <v>2015</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G15" s="1">
-        <v>0</v>
-      </c>
-      <c r="H15" s="1">
-        <v>0</v>
-      </c>
-      <c r="J15" s="1">
-        <v>0</v>
-      </c>
-      <c r="K15" s="1">
+      <c r="G16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
         <v>1</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="L16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M16" s="1">
         <v>4</v>
       </c>
-      <c r="O15" s="1">
-        <v>0</v>
-      </c>
-      <c r="P15" s="1" t="s">
+      <c r="O16" s="1">
+        <v>0</v>
+      </c>
+      <c r="P16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q16" s="1">
         <v>38400</v>
       </c>
-      <c r="R15" s="1">
-        <v>0</v>
-      </c>
-      <c r="S15" s="1">
+      <c r="R16" s="1">
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
         <v>3</v>
       </c>
-      <c r="T15" s="1">
-        <v>0</v>
-      </c>
-      <c r="U15" s="1">
-        <v>0</v>
-      </c>
+      <c r="T16" s="1">
+        <v>0</v>
+      </c>
+      <c r="U16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>